<commit_message>
Extend 领航1号 sheet/chart back to 2026-03-02
- data/lh_nav_history.json: archive of 领航1号 daily NAV from 2026-03-01
  through 2026-04-10 (user-supplied)
- pipeline/combined.py: 领航1号's sheet and the dual-axis chart now use the
  union of historical trading days (filtered by CSI 500 cache) and sample
  dates, so the cumulative-excess baseline is the strategy's earliest
  trading day instead of the first sample date. Other product sheets are
  unchanged.

https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260519_table.xlsx
+++ b/output/20260410_20260519_table.xlsx
@@ -218,7 +218,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="27708225" cy="9124950"/>
+    <ext cx="44510325" cy="9124950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2628,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:BB9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2657,6 +2657,34 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
+    <col width="12" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
+    <col width="12" customWidth="1" min="53" max="53"/>
+    <col width="12" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2667,125 +2695,265 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>2026-04-13</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>2026-04-17</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>2026-04-23</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>2026-04-24</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
@@ -2798,78 +2966,162 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.9991</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.9991</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.9982</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1.0034</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1.0003</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1.007</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>1.0067</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.9985000000000001</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.9966</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>0.9979</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>0.9818</v>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>0.9929</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>0.9723000000000001</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>0.9656</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>0.9297</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>0.9582000000000001</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>0.9755</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>0.9762999999999999</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>0.9806</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>0.9595</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>0.9845</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>0.9594</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>1.0007</v>
+      </c>
+      <c r="AD2" s="3" t="n">
         <v>1.0192</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="AE2" s="3" t="n">
         <v>1.0216</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="AF2" s="3" t="n">
         <v>1.0385</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="AG2" s="3" t="n">
         <v>1.0392</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="AH2" s="3" t="n">
         <v>1.0634</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="AI2" s="3" t="n">
         <v>1.0627</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="AJ2" s="3" t="n">
         <v>1.0668</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="AK2" s="3" t="n">
         <v>1.0673</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="AL2" s="3" t="n">
         <v>1.0822</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="AM2" s="3" t="n">
         <v>1.0609</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="AN2" s="3" t="n">
         <v>1.0638</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="AO2" s="3" t="n">
         <v>1.0714</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="AP2" s="3" t="n">
         <v>1.0638</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="AQ2" s="3" t="n">
         <v>1.0964</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="AR2" s="3" t="n">
         <v>1.0972</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="AS2" s="3" t="n">
         <v>1.1419</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="AT2" s="3" t="n">
         <v>1.1576</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="AU2" s="3" t="n">
         <v>1.1465</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="AV2" s="3" t="n">
         <v>1.1765</v>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="AW2" s="3" t="n">
         <v>1.1697</v>
       </c>
-      <c r="V2" s="3" t="n">
+      <c r="AX2" s="3" t="n">
         <v>1.1915</v>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="AY2" s="3" t="n">
         <v>1.1558</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="AZ2" s="3" t="n">
         <v>1.1322</v>
       </c>
-      <c r="Y2" s="3" t="n">
+      <c r="BA2" s="3" t="n">
         <v>1.1332</v>
       </c>
-      <c r="Z2" s="3" t="n">
+      <c r="BB2" s="3" t="n">
         <v>1.1382</v>
       </c>
     </row>
@@ -2879,79 +3131,107 @@
           <t>今年以来收益率</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
+      <c r="T3" s="4" t="n"/>
+      <c r="U3" s="4" t="n"/>
+      <c r="V3" s="4" t="n"/>
+      <c r="W3" s="4" t="n"/>
+      <c r="X3" s="4" t="n"/>
+      <c r="Y3" s="4" t="n"/>
+      <c r="Z3" s="4" t="n"/>
+      <c r="AA3" s="4" t="n"/>
+      <c r="AB3" s="4" t="n"/>
+      <c r="AC3" s="4" t="n"/>
+      <c r="AD3" s="4" t="n">
         <v>0.0191</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="AE3" s="4" t="n">
         <v>0.0216</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="AF3" s="4" t="n">
         <v>0.0385</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="AG3" s="4" t="n">
         <v>0.0392</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="AH3" s="4" t="n">
         <v>0.0633</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="AI3" s="4" t="n">
         <v>0.0626</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="AJ3" s="4" t="n">
         <v>0.0668</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="AK3" s="4" t="n">
         <v>0.0673</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="AL3" s="4" t="n">
         <v>0.08220000000000001</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="AM3" s="4" t="n">
         <v>0.0609</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="AN3" s="4" t="n">
         <v>0.0638</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="AO3" s="4" t="n">
         <v>0.07139999999999999</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="AP3" s="4" t="n">
         <v>0.0638</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="AQ3" s="4" t="n">
         <v>0.0964</v>
       </c>
-      <c r="P3" s="4" t="n">
+      <c r="AR3" s="4" t="n">
         <v>0.09710000000000001</v>
       </c>
-      <c r="Q3" s="4" t="n">
+      <c r="AS3" s="4" t="n">
         <v>0.1419</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="AT3" s="4" t="n">
         <v>0.1576</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="AU3" s="4" t="n">
         <v>0.1465</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="AV3" s="4" t="n">
         <v>0.1765</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="AW3" s="4" t="n">
         <v>0.1697</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="AX3" s="4" t="n">
         <v>0.1915</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="AY3" s="4" t="n">
         <v>0.1558</v>
       </c>
-      <c r="X3" s="4" t="n">
+      <c r="AZ3" s="4" t="n">
         <v>0.1322</v>
       </c>
-      <c r="Y3" s="4" t="n">
+      <c r="BA3" s="4" t="n">
         <v>0.1332</v>
       </c>
-      <c r="Z3" s="4" t="n">
+      <c r="BB3" s="4" t="n">
         <v>0.1382</v>
       </c>
     </row>
@@ -2961,79 +3241,107 @@
           <t>单日单位净值变动</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
+      <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="5" t="n"/>
+      <c r="R4" s="5" t="n"/>
+      <c r="S4" s="5" t="n"/>
+      <c r="T4" s="5" t="n"/>
+      <c r="U4" s="5" t="n"/>
+      <c r="V4" s="5" t="n"/>
+      <c r="W4" s="5" t="n"/>
+      <c r="X4" s="5" t="n"/>
+      <c r="Y4" s="5" t="n"/>
+      <c r="Z4" s="5" t="n"/>
+      <c r="AA4" s="5" t="n"/>
+      <c r="AB4" s="5" t="n"/>
+      <c r="AC4" s="5" t="n"/>
+      <c r="AD4" s="5" t="n">
         <v>0.0185</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="AE4" s="5" t="n">
         <v>0.0025</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="AF4" s="5" t="n">
         <v>0.0165</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="AG4" s="5" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="AH4" s="5" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="AI4" s="5" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="AJ4" s="5" t="n">
         <v>0.004</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="AK4" s="5" t="n">
         <v>0.0005</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="AL4" s="5" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="AM4" s="5" t="n">
         <v>-0.0197</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="AN4" s="5" t="n">
         <v>0.0027</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="AO4" s="5" t="n">
         <v>0.0072</v>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="AP4" s="5" t="n">
         <v>-0.0071</v>
       </c>
-      <c r="O4" s="5" t="n">
+      <c r="AQ4" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="P4" s="5" t="n">
+      <c r="AR4" s="5" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="AS4" s="5" t="n">
         <v>0.04099999999999999</v>
       </c>
-      <c r="R4" s="5" t="n">
+      <c r="AT4" s="5" t="n">
         <v>0.0137</v>
       </c>
-      <c r="S4" s="5" t="n">
+      <c r="AU4" s="5" t="n">
         <v>-0.009599999999999999</v>
       </c>
-      <c r="T4" s="5" t="n">
+      <c r="AV4" s="5" t="n">
         <v>0.0263</v>
       </c>
-      <c r="U4" s="5" t="n">
+      <c r="AW4" s="5" t="n">
         <v>-0.0058</v>
       </c>
-      <c r="V4" s="5" t="n">
+      <c r="AX4" s="5" t="n">
         <v>0.0186</v>
       </c>
-      <c r="W4" s="5" t="n">
+      <c r="AY4" s="5" t="n">
         <v>-0.03</v>
       </c>
-      <c r="X4" s="5" t="n">
+      <c r="AZ4" s="5" t="n">
         <v>-0.0204</v>
       </c>
-      <c r="Y4" s="5" t="n">
+      <c r="BA4" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="Z4" s="5" t="n">
+      <c r="BB4" s="5" t="n">
         <v>0.0044</v>
       </c>
     </row>
@@ -3044,78 +3352,162 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
+        <v>4728.6688</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>4655.8962</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>4602.6247</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>4647.6921</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>4660.439</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>4615.4551</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>4674.7562</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>4704.4959</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>4687.5601</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>4669.14</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>4671.5591</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>4637.4392</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>4658.3324</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>4583.2511</v>
+      </c>
+      <c r="P5" s="7" t="n">
+        <v>4567.0179</v>
+      </c>
+      <c r="Q5" s="7" t="n">
+        <v>4417.9971</v>
+      </c>
+      <c r="R5" s="7" t="n">
+        <v>4474.7224</v>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>4537.4656</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>4477.5343</v>
+      </c>
+      <c r="U5" s="7" t="n">
+        <v>4502.5698</v>
+      </c>
+      <c r="V5" s="7" t="n">
+        <v>4491.95</v>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>4450.0493</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>4526.0668</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>4478.9141</v>
+      </c>
+      <c r="Z5" s="7" t="n">
+        <v>4440.7889</v>
+      </c>
+      <c r="AA5" s="7" t="n">
+        <v>4440.6162</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>4595.556</v>
+      </c>
+      <c r="AC5" s="7" t="n">
+        <v>4566.2237</v>
+      </c>
+      <c r="AD5" s="7" t="n">
         <v>4636.5655</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="AE5" s="7" t="n">
         <v>4646.1546</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="AF5" s="7" t="n">
         <v>4701.2837</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="AG5" s="7" t="n">
         <v>4685.2464</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="AH5" s="7" t="n">
         <v>4736.6077</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="AI5" s="7" t="n">
         <v>4728.6716</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="AJ5" s="7" t="n">
         <v>4757.4419</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="AK5" s="7" t="n">
         <v>4767.997</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="AL5" s="7" t="n">
         <v>4799.627</v>
       </c>
-      <c r="K5" s="7" t="n">
+      <c r="AM5" s="7" t="n">
         <v>4786.3273</v>
       </c>
-      <c r="L5" s="7" t="n">
+      <c r="AN5" s="7" t="n">
         <v>4769.3688</v>
       </c>
-      <c r="M5" s="7" t="n">
+      <c r="AO5" s="7" t="n">
         <v>4770.9469</v>
       </c>
-      <c r="N5" s="7" t="n">
+      <c r="AP5" s="7" t="n">
         <v>4758.2083</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="AQ5" s="7" t="n">
         <v>4810.3468</v>
       </c>
-      <c r="P5" s="7" t="n">
+      <c r="AR5" s="7" t="n">
         <v>4807.3069</v>
       </c>
-      <c r="Q5" s="7" t="n">
+      <c r="AS5" s="7" t="n">
         <v>4877.0932</v>
       </c>
-      <c r="R5" s="7" t="n">
+      <c r="AT5" s="7" t="n">
         <v>4900.5098</v>
       </c>
-      <c r="S5" s="7" t="n">
+      <c r="AU5" s="7" t="n">
         <v>4871.9122</v>
       </c>
-      <c r="T5" s="7" t="n">
+      <c r="AV5" s="7" t="n">
         <v>4951.8366</v>
       </c>
-      <c r="U5" s="7" t="n">
+      <c r="AW5" s="7" t="n">
         <v>4948.0465</v>
       </c>
-      <c r="V5" s="7" t="n">
+      <c r="AX5" s="7" t="n">
         <v>4998.3417</v>
       </c>
-      <c r="W5" s="7" t="n">
+      <c r="AY5" s="7" t="n">
         <v>4914.5971</v>
       </c>
-      <c r="X5" s="7" t="n">
+      <c r="AZ5" s="7" t="n">
         <v>4859.5927</v>
       </c>
-      <c r="Y5" s="7" t="n">
+      <c r="BA5" s="7" t="n">
         <v>4833.5237</v>
       </c>
-      <c r="Z5" s="7" t="n">
+      <c r="BB5" s="7" t="n">
         <v>4852.8832</v>
       </c>
     </row>
@@ -3126,78 +3518,162 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
+        <v>8658.3336</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>8281.6139</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>8248.945</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>8309.1713</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>8360.334699999999</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>8279.481100000001</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>8410.303</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>8403.329599999999</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>8359.472100000001</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>8239.798000000001</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>8185.152</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>8016.0262</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>8096.4276</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>7877.09</v>
+      </c>
+      <c r="P6" s="7" t="n">
+        <v>7760.0365</v>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>7440.7451</v>
+      </c>
+      <c r="R6" s="7" t="n">
+        <v>7597.3732</v>
+      </c>
+      <c r="S6" s="7" t="n">
+        <v>7767.6654</v>
+      </c>
+      <c r="T6" s="7" t="n">
+        <v>7642.1302</v>
+      </c>
+      <c r="U6" s="7" t="n">
+        <v>7737.6144</v>
+      </c>
+      <c r="V6" s="7" t="n">
+        <v>7753.7234</v>
+      </c>
+      <c r="W6" s="7" t="n">
+        <v>7617.3262</v>
+      </c>
+      <c r="X6" s="7" t="n">
+        <v>7750.0924</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>7605.2932</v>
+      </c>
+      <c r="Z6" s="7" t="n">
+        <v>7534.938</v>
+      </c>
+      <c r="AA6" s="7" t="n">
+        <v>7571.1106</v>
+      </c>
+      <c r="AB6" s="7" t="n">
+        <v>7945.1527</v>
+      </c>
+      <c r="AC6" s="7" t="n">
+        <v>7898.6329</v>
+      </c>
+      <c r="AD6" s="7" t="n">
         <v>7969.3646</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="AE6" s="7" t="n">
         <v>7967.697</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="AF6" s="7" t="n">
         <v>8088.5687</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="AG6" s="7" t="n">
         <v>8044.0773</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="AH6" s="7" t="n">
         <v>8180.0815</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="AI6" s="7" t="n">
         <v>8214.1939</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="AJ6" s="7" t="n">
         <v>8290.0224</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="AK6" s="7" t="n">
         <v>8270.3266</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="AL6" s="7" t="n">
         <v>8376.1808</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="AM6" s="7" t="n">
         <v>8295.207</v>
       </c>
-      <c r="L6" s="7" t="n">
+      <c r="AN6" s="7" t="n">
         <v>8247.875899999999</v>
       </c>
-      <c r="M6" s="7" t="n">
+      <c r="AO6" s="7" t="n">
         <v>8299.0486</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="AP6" s="7" t="n">
         <v>8203.9614</v>
       </c>
-      <c r="O6" s="7" t="n">
+      <c r="AQ6" s="7" t="n">
         <v>8342.421700000001</v>
       </c>
-      <c r="P6" s="7" t="n">
+      <c r="AR6" s="7" t="n">
         <v>8349.508099999999</v>
       </c>
-      <c r="Q6" s="7" t="n">
+      <c r="AS6" s="7" t="n">
         <v>8588.439899999999</v>
       </c>
-      <c r="R6" s="7" t="n">
+      <c r="AT6" s="7" t="n">
         <v>8696.7989</v>
       </c>
-      <c r="S6" s="7" t="n">
+      <c r="AU6" s="7" t="n">
         <v>8694.170899999999</v>
       </c>
-      <c r="T6" s="7" t="n">
+      <c r="AV6" s="7" t="n">
         <v>8839.7415</v>
       </c>
-      <c r="U6" s="7" t="n">
+      <c r="AW6" s="7" t="n">
         <v>8785.9791</v>
       </c>
-      <c r="V6" s="7" t="n">
+      <c r="AX6" s="7" t="n">
         <v>8918.239</v>
       </c>
-      <c r="W6" s="7" t="n">
+      <c r="AY6" s="7" t="n">
         <v>8670.1574</v>
       </c>
-      <c r="X6" s="7" t="n">
+      <c r="AZ6" s="7" t="n">
         <v>8536.3444</v>
       </c>
-      <c r="Y6" s="7" t="n">
+      <c r="BA6" s="7" t="n">
         <v>8554.2372</v>
       </c>
-      <c r="Z6" s="7" t="n">
+      <c r="BB6" s="7" t="n">
         <v>8627.946099999999</v>
       </c>
     </row>
@@ -3305,6 +3781,118 @@
       </c>
       <c r="Z7" s="9">
         <f>(Z2/$B$2-1)-(Z6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AA7" s="9">
+        <f>(AA2/$B$2-1)-(AA6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AB7" s="9">
+        <f>(AB2/$B$2-1)-(AB6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="9">
+        <f>(AC2/$B$2-1)-(AC6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AD7" s="9">
+        <f>(AD2/$B$2-1)-(AD6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AE7" s="9">
+        <f>(AE2/$B$2-1)-(AE6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AF7" s="9">
+        <f>(AF2/$B$2-1)-(AF6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AG7" s="9">
+        <f>(AG2/$B$2-1)-(AG6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AH7" s="9">
+        <f>(AH2/$B$2-1)-(AH6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AI7" s="9">
+        <f>(AI2/$B$2-1)-(AI6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="9">
+        <f>(AJ2/$B$2-1)-(AJ6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AK7" s="9">
+        <f>(AK2/$B$2-1)-(AK6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AL7" s="9">
+        <f>(AL2/$B$2-1)-(AL6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AM7" s="9">
+        <f>(AM2/$B$2-1)-(AM6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AN7" s="9">
+        <f>(AN2/$B$2-1)-(AN6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AO7" s="9">
+        <f>(AO2/$B$2-1)-(AO6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AP7" s="9">
+        <f>(AP2/$B$2-1)-(AP6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AQ7" s="9">
+        <f>(AQ2/$B$2-1)-(AQ6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AR7" s="9">
+        <f>(AR2/$B$2-1)-(AR6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AS7" s="9">
+        <f>(AS2/$B$2-1)-(AS6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AT7" s="9">
+        <f>(AT2/$B$2-1)-(AT6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AU7" s="9">
+        <f>(AU2/$B$2-1)-(AU6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AV7" s="9">
+        <f>(AV2/$B$2-1)-(AV6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AW7" s="9">
+        <f>(AW2/$B$2-1)-(AW6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AX7" s="9">
+        <f>(AX2/$B$2-1)-(AX6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AY7" s="9">
+        <f>(AY2/$B$2-1)-(AY6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="AZ7" s="9">
+        <f>(AZ2/$B$2-1)-(AZ6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="BA7" s="9">
+        <f>(BA2/$B$2-1)-(BA6/$B$6-1)</f>
+        <v/>
+      </c>
+      <c r="BB7" s="9">
+        <f>(BB2/$B$2-1)-(BB6/$B$6-1)</f>
         <v/>
       </c>
     </row>

</xml_diff>